<commit_message>
feat(perf-strategica): consuntivazione referente, composite, visibilita' Interrogazione
- saveIndicatorConsuntivo: workEffortId scheda + data fine periodo (valore ora
  visibile nei report legacy), scoping per-UO, idempotenza (servicedef export + controller)
- executePerformFindBSWorkEffortRootInqy: DIR_SAN/DIR_AMM vedono tutte le schede
- POST_IMPORT_PARAMETRI_COMPOSITE.sql: 5 indicatori composite (rapporto/variazione/somma)
  + wrapper SETUP_POST_IMPORT.sql; fasce/parametri generati; profili DIR_SAN/AMM
- card indicatore Cardarelli (formula parlante), template import riconciliati,
  tooling generatori + verifica-import (Playwright)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/script/templates/WeRootInterface_BS.xlsx
+++ b/script/templates/WeRootInterface_BS.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Servizio Ispettivo</t>
+          <t>Obiettivo Performance Strategica UOC Gestione Risorse Umane</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Obiettivo Performance Strategica UOC Investimenti e Energy Management</t>
+          <t>Obiettivo Performance Strategica UOC Gestione Risorse Tecniche</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">

</xml_diff>